<commit_message>
feat: configure Strategic Sourcing LGE eMMC R&R for Nam Seohyeon (Sales) and Lee Hayoung (CS)
</commit_message>
<xml_diff>
--- a/input/RAmos_조직도_업무스킬_양식.xlsx
+++ b/input/RAmos_조직도_업무스킬_양식.xlsx
@@ -1914,9 +1914,21 @@
           <t>shnam1228@ramostek.com</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>전략소싱팀 LGE eMMC 영업 담당, 고객사 소통, 공급 조율</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>eMMC 5.1, Flash</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>LGE 고객 영업, 납기/단가 조율, 계약 관리</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1944,9 +1956,21 @@
           <t>lhyduddlgk@ramostek.com</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>전략소싱팀 LGE eMMC CS 담당, 고객 불량 클레임 1차 접수 및 소통</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>eMMC 5.1, Flash</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>LGE 고객 CS, 초동 접수, 부적합 소통, 클레임 채널</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: enforce LGE DTV eMMC business model with Inked NAND die domain context
</commit_message>
<xml_diff>
--- a/input/RAmos_조직도_업무스킬_양식.xlsx
+++ b/input/RAmos_조직도_업무스킬_양식.xlsx
@@ -1916,17 +1916,17 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>전략소싱팀 LGE eMMC 영업 담당, 고객사 소통, 공급 조율</t>
+          <t>전략소싱팀 LGE DTV eMMC 영업 주관, 고객사 소통, 공급 계약</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>eMMC 5.1, Flash</t>
+          <t>LGE DTV eMMC 5.1 (Inked NAND 적용)</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>LGE 고객 영업, 납기/단가 조율, 계약 관리</t>
+          <t>LGE DTV 영업 대응, 납기/단가 조율, 계약 관리</t>
         </is>
       </c>
     </row>
@@ -1958,17 +1958,17 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>전략소싱팀 LGE eMMC CS 담당, 고객 불량 클레임 1차 접수 및 소통</t>
+          <t>전략소싱팀 LGE DTV eMMC CS 주관, 부적합 클레임 1차 접수 및 소통</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>eMMC 5.1, Flash</t>
+          <t>LGE DTV eMMC 5.1 (Inked NAND 적용)</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>LGE 고객 CS, 초동 접수, 부적합 소통, 클레임 채널</t>
+          <t>LGE DTV CS 대응, 초동 접수, 부적합 소통, 클레임 채널</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: isolate customer-facing LGE claim terminology from internal Inked NAND FA analysis
</commit_message>
<xml_diff>
--- a/input/RAmos_조직도_업무스킬_양식.xlsx
+++ b/input/RAmos_조직도_업무스킬_양식.xlsx
@@ -1220,17 +1220,17 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Physical FA / 불량 분석 총괄, 시각 증거 검증</t>
+          <t>Physical FA / eMMC 불량 분석 총괄, 시각 증거 검증</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>eMMC, Flash</t>
+          <t>LGE DTV eMMC 5.1 (BGA153)</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>SEM 단면분석, Decap, X-Ray, BGA 쇼트</t>
+          <t>SEM 단면분석, Decap, Inked NAND Die 셀 마진 분석, EDS Inking 맵 대조</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>LGE DTV eMMC 5.1 (Inked NAND 적용)</t>
+          <t>LGE DTV eMMC 5.1 (BGA153)</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>LGE DTV eMMC 5.1 (Inked NAND 적용)</t>
+          <t>LGE DTV eMMC 5.1 (BGA153)</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">

</xml_diff>